<commit_message>
Update OUTPUT_DIR to encoded_files, fix README and gitignore
</commit_message>
<xml_diff>
--- a/script/qp_analysis_report.xlsx
+++ b/script/qp_analysis_report.xlsx
@@ -447,7 +447,7 @@
     <from>
       <col>5</col>
       <colOff>0</colOff>
-      <row>26</row>
+      <row>22</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7200000" cy="4320000"/>
@@ -790,7 +790,7 @@
         <v>17300.5341796875</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>121.48</v>
+        <v>221.52</v>
       </c>
     </row>
     <row r="3">
@@ -801,7 +801,7 @@
         <v>16334.3310546875</v>
       </c>
       <c r="C3" s="7" t="n">
-        <v>117.92</v>
+        <v>192.34</v>
       </c>
     </row>
     <row r="4">
@@ -812,7 +812,7 @@
         <v>15281.0888671875</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>89.51000000000001</v>
+        <v>196.31</v>
       </c>
     </row>
     <row r="5">
@@ -823,7 +823,7 @@
         <v>14316.8251953125</v>
       </c>
       <c r="C5" s="7" t="n">
-        <v>77.11</v>
+        <v>188.69</v>
       </c>
     </row>
     <row r="6">
@@ -834,7 +834,7 @@
         <v>13246.4365234375</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>67.44</v>
+        <v>196.78</v>
       </c>
     </row>
     <row r="7">
@@ -845,7 +845,7 @@
         <v>12104.7373046875</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>49.4</v>
+        <v>192.44</v>
       </c>
     </row>
     <row r="8">
@@ -856,7 +856,7 @@
         <v>11023.2099609375</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>54.12</v>
+        <v>195.66</v>
       </c>
     </row>
     <row r="9">
@@ -867,7 +867,7 @@
         <v>9840.18359375</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>72.89</v>
+        <v>204.34</v>
       </c>
     </row>
     <row r="10">
@@ -878,7 +878,7 @@
         <v>8761.6435546875</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>83.23999999999999</v>
+        <v>197.5</v>
       </c>
     </row>
     <row r="11">
@@ -889,7 +889,7 @@
         <v>7721.9111328125</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>95.39</v>
+        <v>212.44</v>
       </c>
     </row>
     <row r="12">
@@ -900,7 +900,7 @@
         <v>6763.0888671875</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>98.20999999999999</v>
+        <v>224.85</v>
       </c>
     </row>
     <row r="13">
@@ -911,7 +911,7 @@
         <v>5895.84375</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>86.09999999999999</v>
+        <v>238.24</v>
       </c>
     </row>
     <row r="14">
@@ -922,7 +922,7 @@
         <v>5104.1201171875</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>107.7</v>
+        <v>238.93</v>
       </c>
     </row>
     <row r="15">
@@ -933,7 +933,7 @@
         <v>4360.9052734375</v>
       </c>
       <c r="C15" s="7" t="n">
-        <v>115.04</v>
+        <v>231.65</v>
       </c>
     </row>
     <row r="16">
@@ -944,7 +944,7 @@
         <v>3714.1083984375</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>128.09</v>
+        <v>260.57</v>
       </c>
     </row>
     <row r="17">
@@ -955,7 +955,7 @@
         <v>3145.8984375</v>
       </c>
       <c r="C17" s="7" t="n">
-        <v>141.85</v>
+        <v>290.63</v>
       </c>
     </row>
     <row r="18">
@@ -966,7 +966,7 @@
         <v>2670.2919921875</v>
       </c>
       <c r="C18" s="4" t="n">
-        <v>151.56</v>
+        <v>308.12</v>
       </c>
     </row>
     <row r="19">
@@ -977,7 +977,7 @@
         <v>2270.1669921875</v>
       </c>
       <c r="C19" s="7" t="n">
-        <v>148.84</v>
+        <v>319.65</v>
       </c>
     </row>
     <row r="20">
@@ -988,7 +988,7 @@
         <v>1931.1689453125</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>165.84</v>
+        <v>322.35</v>
       </c>
     </row>
     <row r="21">
@@ -999,7 +999,7 @@
         <v>1628.8505859375</v>
       </c>
       <c r="C21" s="7" t="n">
-        <v>169.78</v>
+        <v>354.86</v>
       </c>
     </row>
     <row r="22">
@@ -1010,7 +1010,7 @@
         <v>1394.0234375</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>178.36</v>
+        <v>348.87</v>
       </c>
     </row>
     <row r="23">
@@ -1021,7 +1021,7 @@
         <v>1185.23046875</v>
       </c>
       <c r="C23" s="7" t="n">
-        <v>179.55</v>
+        <v>387.11</v>
       </c>
     </row>
     <row r="24">
@@ -1032,7 +1032,7 @@
         <v>1015.263671875</v>
       </c>
       <c r="C24" s="4" t="n">
-        <v>154.23</v>
+        <v>373.24</v>
       </c>
     </row>
     <row r="25">
@@ -1043,7 +1043,7 @@
         <v>867.7412109375</v>
       </c>
       <c r="C25" s="7" t="n">
-        <v>185.85</v>
+        <v>371.65</v>
       </c>
     </row>
     <row r="26">
@@ -1054,7 +1054,7 @@
         <v>750.5966796875</v>
       </c>
       <c r="C26" s="4" t="n">
-        <v>208.27</v>
+        <v>417.74</v>
       </c>
     </row>
     <row r="27">
@@ -1065,7 +1065,7 @@
         <v>644.69921875</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>201.1</v>
+        <v>445.15</v>
       </c>
     </row>
     <row r="28">
@@ -1076,7 +1076,7 @@
         <v>558.2568359375</v>
       </c>
       <c r="C28" s="4" t="n">
-        <v>239.95</v>
+        <v>464.82</v>
       </c>
     </row>
     <row r="29">
@@ -1087,7 +1087,7 @@
         <v>481.7470703125</v>
       </c>
       <c r="C29" s="7" t="n">
-        <v>245.95</v>
+        <v>476.97</v>
       </c>
     </row>
     <row r="30">
@@ -1098,7 +1098,7 @@
         <v>419.0302734375</v>
       </c>
       <c r="C30" s="4" t="n">
-        <v>240.19</v>
+        <v>493.84</v>
       </c>
     </row>
     <row r="31">
@@ -1109,7 +1109,7 @@
         <v>366.5224609375</v>
       </c>
       <c r="C31" s="7" t="n">
-        <v>231.08</v>
+        <v>515.52</v>
       </c>
     </row>
     <row r="32">
@@ -1120,7 +1120,7 @@
         <v>321.646484375</v>
       </c>
       <c r="C32" s="4" t="n">
-        <v>279.16</v>
+        <v>525.55</v>
       </c>
     </row>
     <row r="33">
@@ -1131,7 +1131,7 @@
         <v>283.013671875</v>
       </c>
       <c r="C33" s="7" t="n">
-        <v>303.35</v>
+        <v>539.7</v>
       </c>
     </row>
     <row r="34">
@@ -1142,7 +1142,7 @@
         <v>250.216796875</v>
       </c>
       <c r="C34" s="4" t="n">
-        <v>339.92</v>
+        <v>572.04</v>
       </c>
     </row>
     <row r="35">
@@ -1153,7 +1153,7 @@
         <v>221.51953125</v>
       </c>
       <c r="C35" s="7" t="n">
-        <v>311.98</v>
+        <v>590.14</v>
       </c>
     </row>
     <row r="36">
@@ -1164,7 +1164,7 @@
         <v>196.763671875</v>
       </c>
       <c r="C36" s="4" t="n">
-        <v>338.93</v>
+        <v>634.74</v>
       </c>
     </row>
     <row r="37">
@@ -1175,7 +1175,7 @@
         <v>176.158203125</v>
       </c>
       <c r="C37" s="7" t="n">
-        <v>363.18</v>
+        <v>569.74</v>
       </c>
     </row>
     <row r="38">
@@ -1186,7 +1186,7 @@
         <v>158.0068359375</v>
       </c>
       <c r="C38" s="4" t="n">
-        <v>382.26</v>
+        <v>598.45</v>
       </c>
     </row>
     <row r="39">
@@ -1197,7 +1197,7 @@
         <v>140.12109375</v>
       </c>
       <c r="C39" s="7" t="n">
-        <v>415.08</v>
+        <v>685.85</v>
       </c>
     </row>
     <row r="40">
@@ -1208,7 +1208,7 @@
         <v>127.564453125</v>
       </c>
       <c r="C40" s="4" t="n">
-        <v>409.28</v>
+        <v>721.85</v>
       </c>
     </row>
     <row r="41">
@@ -1219,7 +1219,7 @@
         <v>114.728515625</v>
       </c>
       <c r="C41" s="7" t="n">
-        <v>330.18</v>
+        <v>727.03</v>
       </c>
     </row>
     <row r="42">
@@ -1230,7 +1230,7 @@
         <v>103.744140625</v>
       </c>
       <c r="C42" s="4" t="n">
-        <v>446.17</v>
+        <v>777.02</v>
       </c>
     </row>
     <row r="43">
@@ -1241,7 +1241,7 @@
         <v>93.1904296875</v>
       </c>
       <c r="C43" s="7" t="n">
-        <v>452.46</v>
+        <v>785.45</v>
       </c>
     </row>
     <row r="44">
@@ -1252,7 +1252,7 @@
         <v>85.7353515625</v>
       </c>
       <c r="C44" s="4" t="n">
-        <v>443.39</v>
+        <v>806.87</v>
       </c>
     </row>
     <row r="45">
@@ -1263,7 +1263,7 @@
         <v>77.83203125</v>
       </c>
       <c r="C45" s="7" t="n">
-        <v>469.83</v>
+        <v>754.12</v>
       </c>
     </row>
     <row r="46">
@@ -1274,7 +1274,7 @@
         <v>71.4267578125</v>
       </c>
       <c r="C46" s="4" t="n">
-        <v>478.81</v>
+        <v>807</v>
       </c>
     </row>
     <row r="47">
@@ -1285,7 +1285,7 @@
         <v>65.427734375</v>
       </c>
       <c r="C47" s="7" t="n">
-        <v>483.05</v>
+        <v>833.49</v>
       </c>
     </row>
     <row r="48">
@@ -1296,7 +1296,7 @@
         <v>59.7216796875</v>
       </c>
       <c r="C48" s="4" t="n">
-        <v>382.31</v>
+        <v>882</v>
       </c>
     </row>
     <row r="49">
@@ -1307,7 +1307,7 @@
         <v>54.06640625</v>
       </c>
       <c r="C49" s="7" t="n">
-        <v>510.41</v>
+        <v>857.33</v>
       </c>
     </row>
     <row r="50">
@@ -1318,7 +1318,7 @@
         <v>50.2138671875</v>
       </c>
       <c r="C50" s="4" t="n">
-        <v>508.42</v>
+        <v>905.22</v>
       </c>
     </row>
     <row r="51">
@@ -1329,7 +1329,7 @@
         <v>45.4912109375</v>
       </c>
       <c r="C51" s="7" t="n">
-        <v>520.2</v>
+        <v>925.13</v>
       </c>
     </row>
     <row r="52">
@@ -1340,7 +1340,7 @@
         <v>41.83984375</v>
       </c>
       <c r="C52" s="4" t="n">
-        <v>536.34</v>
+        <v>918.09</v>
       </c>
     </row>
   </sheetData>

</xml_diff>